<commit_message>
Versión sencilla: agrega tabla dinámica con filtros y registro de tareas
Nueva hoja REGISTRO DE TAREAS (una tarea por fila, como tabla de Excel)
que alimenta la TABLA DINÁMICA: filtros de Mes y Tipo de actividad,
filas por Asignatura y columnas por Estado de entrega. La sección 4 de
DATOS ahora cuenta las tareas desde ese registro; los resultados del
tablero no cambian.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0134eJ6gavT5KxExpqB4Y73E
</commit_message>
<xml_diff>
--- a/PROYECTO INTEGRADOR · ETAPA 2 · Tablero de control (sencillo).xlsx
+++ b/PROYECTO INTEGRADOR · ETAPA 2 · Tablero de control (sencillo).xlsx
@@ -10,11 +10,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ENCABEZADO" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TABLERO DE CONTROL" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONCLUSIÓN" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DATOS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REFERENCIAS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TABLA DINÁMICA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DATOS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REGISTRO DE TAREAS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REFERENCIAS" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <pivotCaches>
+    <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="1" r:id="rId8"/>
+  </pivotCaches>
 </workbook>
 </file>
 
@@ -119,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -195,6 +200,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -991,6 +1008,529 @@
 </wsDr>
 </file>
 
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" refreshOnLoad="1" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="40" r:id="rId1">
+  <cacheSource type="worksheet">
+    <worksheetSource name="TablaTareas"/>
+  </cacheSource>
+  <cacheFields count="7">
+    <cacheField name="N.º" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsInteger="1" containsNumber="1" containsSemiMixedTypes="0" containsString="0" minValue="1" maxValue="40"/>
+    </cacheField>
+    <cacheField name="Fecha de entrega" uniqueList="1" numFmtId="14" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsDate="1" containsNonDate="0" containsSemiMixedTypes="0" containsString="0" minDate="2026-09-02T00:00:00" maxDate="2026-10-16T00:00:00"/>
+    </cacheField>
+    <cacheField name="Mes" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="2">
+        <s v="Septiembre"/>
+        <s v="Octubre"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Asignatura" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="5">
+        <s v="Matemáticas"/>
+        <s v="Comunicación oral y escrita"/>
+        <s v="Inglés"/>
+        <s v="Tecnologías de información"/>
+        <s v="Desarrollo humano"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Tipo de actividad" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="4">
+        <s v="Tarea"/>
+        <s v="Ejercicios de repaso"/>
+        <s v="Reporte de lectura"/>
+        <s v="Proyecto"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Estado de entrega" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="3">
+        <s v="A tiempo"/>
+        <s v="Con retraso"/>
+        <s v="No entregada"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Calificación" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1" containsNumber="1" containsString="0" minValue="6.3" maxValue="9.9"/>
+    </cacheField>
+  </cacheFields>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40">
+  <r>
+    <n v="1"/>
+    <d v="2026-09-02T00:00:00"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="7.3"/>
+  </r>
+  <r>
+    <n v="2"/>
+    <d v="2026-09-03T00:00:00"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="8.9"/>
+  </r>
+  <r>
+    <n v="3"/>
+    <d v="2026-09-04T00:00:00"/>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="7.9"/>
+  </r>
+  <r>
+    <n v="4"/>
+    <d v="2026-09-05T00:00:00"/>
+    <x v="0"/>
+    <x v="3"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="8.699999999999999"/>
+  </r>
+  <r>
+    <n v="5"/>
+    <d v="2026-09-06T00:00:00"/>
+    <x v="0"/>
+    <x v="4"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="9.300000000000001"/>
+  </r>
+  <r>
+    <n v="6"/>
+    <d v="2026-09-06T00:00:00"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="6.6"/>
+  </r>
+  <r>
+    <n v="7"/>
+    <d v="2026-09-09T00:00:00"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="9.199999999999999"/>
+  </r>
+  <r>
+    <n v="8"/>
+    <d v="2026-09-09T00:00:00"/>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="7.2"/>
+  </r>
+  <r>
+    <n v="9"/>
+    <d v="2026-09-10T00:00:00"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="2"/>
+    <m/>
+  </r>
+  <r>
+    <n v="10"/>
+    <d v="2026-09-11T00:00:00"/>
+    <x v="0"/>
+    <x v="3"/>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="8"/>
+  </r>
+  <r>
+    <n v="11"/>
+    <d v="2026-09-14T00:00:00"/>
+    <x v="0"/>
+    <x v="4"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="9.6"/>
+  </r>
+  <r>
+    <n v="12"/>
+    <d v="2026-09-14T00:00:00"/>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="0"/>
+    <x v="2"/>
+    <m/>
+  </r>
+  <r>
+    <n v="13"/>
+    <d v="2026-09-14T00:00:00"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="1"/>
+    <n v="6.3"/>
+  </r>
+  <r>
+    <n v="14"/>
+    <d v="2026-09-15T00:00:00"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="9.5"/>
+  </r>
+  <r>
+    <n v="15"/>
+    <d v="2026-09-17T00:00:00"/>
+    <x v="0"/>
+    <x v="3"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="9.300000000000001"/>
+  </r>
+  <r>
+    <n v="16"/>
+    <d v="2026-09-18T00:00:00"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="7.6"/>
+  </r>
+  <r>
+    <n v="17"/>
+    <d v="2026-09-19T00:00:00"/>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="7.9"/>
+  </r>
+  <r>
+    <n v="18"/>
+    <d v="2026-09-21T00:00:00"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="8.9"/>
+  </r>
+  <r>
+    <n v="19"/>
+    <d v="2026-09-22T00:00:00"/>
+    <x v="0"/>
+    <x v="4"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="9.9"/>
+  </r>
+  <r>
+    <n v="20"/>
+    <d v="2026-09-22T00:00:00"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="7.9"/>
+  </r>
+  <r>
+    <n v="21"/>
+    <d v="2026-09-23T00:00:00"/>
+    <x v="0"/>
+    <x v="3"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="8.699999999999999"/>
+  </r>
+  <r>
+    <n v="22"/>
+    <d v="2026-09-24T00:00:00"/>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="8.199999999999999"/>
+  </r>
+  <r>
+    <n v="23"/>
+    <d v="2026-09-26T00:00:00"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="7.3"/>
+  </r>
+  <r>
+    <n v="24"/>
+    <d v="2026-09-27T00:00:00"/>
+    <x v="0"/>
+    <x v="1"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="9.199999999999999"/>
+  </r>
+  <r>
+    <n v="25"/>
+    <d v="2026-09-29T00:00:00"/>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="8.5"/>
+  </r>
+  <r>
+    <n v="26"/>
+    <d v="2026-09-29T00:00:00"/>
+    <x v="0"/>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="9"/>
+  </r>
+  <r>
+    <n v="27"/>
+    <d v="2026-09-30T00:00:00"/>
+    <x v="0"/>
+    <x v="4"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="9.300000000000001"/>
+  </r>
+  <r>
+    <n v="28"/>
+    <d v="2026-09-30T00:00:00"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="7.6"/>
+  </r>
+  <r>
+    <n v="29"/>
+    <d v="2026-10-03T00:00:00"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="9.5"/>
+  </r>
+  <r>
+    <n v="30"/>
+    <d v="2026-10-04T00:00:00"/>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="7.9"/>
+  </r>
+  <r>
+    <n v="31"/>
+    <d v="2026-10-04T00:00:00"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="7.9"/>
+  </r>
+  <r>
+    <n v="32"/>
+    <d v="2026-10-05T00:00:00"/>
+    <x v="1"/>
+    <x v="3"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="9.300000000000001"/>
+  </r>
+  <r>
+    <n v="33"/>
+    <d v="2026-10-08T00:00:00"/>
+    <x v="1"/>
+    <x v="4"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="9.6"/>
+  </r>
+  <r>
+    <n v="34"/>
+    <d v="2026-10-08T00:00:00"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="7.3"/>
+  </r>
+  <r>
+    <n v="35"/>
+    <d v="2026-10-09T00:00:00"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="8.9"/>
+  </r>
+  <r>
+    <n v="36"/>
+    <d v="2026-10-09T00:00:00"/>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="8.199999999999999"/>
+  </r>
+  <r>
+    <n v="37"/>
+    <d v="2026-10-11T00:00:00"/>
+    <x v="1"/>
+    <x v="3"/>
+    <x v="1"/>
+    <x v="0"/>
+    <n v="8.699999999999999"/>
+  </r>
+  <r>
+    <n v="38"/>
+    <d v="2026-10-14T00:00:00"/>
+    <x v="1"/>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="0"/>
+    <n v="8.5"/>
+  </r>
+  <r>
+    <n v="39"/>
+    <d v="2026-10-15T00:00:00"/>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="9.199999999999999"/>
+  </r>
+  <r>
+    <n v="40"/>
+    <d v="2026-10-16T00:00:00"/>
+    <x v="1"/>
+    <x v="4"/>
+    <x v="0"/>
+    <x v="0"/>
+    <n v="9.9"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinamicaTareas" cacheId="1" dataOnRows="0" dataCaption="Valores" grandTotalCaption="Total general" showError="0" showMissing="1" updatedVersion="6" minRefreshableVersion="3" asteriskTotals="0" showItems="1" editData="0" disableFieldList="0" showCalcMbrs="1" visualTotals="1" showMultipleLabel="1" showDataDropDown="1" showDrill="1" printDrill="0" showMemberPropertyTips="1" showDataTips="1" enableWizard="1" enableDrill="1" enableFieldProperties="1" preserveFormatting="1" useAutoFormatting="1" pageWrap="0" pageOverThenDown="0" subtotalHiddenItems="0" rowGrandTotals="1" colGrandTotals="1" fieldPrintTitles="0" itemPrintTitles="1" mergeItem="0" showDropZones="1" createdVersion="6" indent="0" showEmptyRow="0" showEmptyCol="0" showHeaders="1" compact="1" outline="1" outlineData="1" compactData="1" published="0" gridDropZones="0" immersive="1" multipleFieldFilters="0" chartFormat="0" rowHeaderCaption="Asignatura" colHeaderCaption="Estado de entrega" fieldListSortAscending="0" mdxSubqueries="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1">
+  <location ref="A7:E14" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
+  <pivotFields count="7">
+    <pivotField dataField="1" showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="1" numFmtId="14" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField axis="axisPage" showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1">
+      <items count="3">
+        <item t="data" sd="1" x="0"/>
+        <item t="data" sd="1" x="1"/>
+        <item t="default" sd="1"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1">
+      <items count="6">
+        <item t="data" sd="1" x="0"/>
+        <item t="data" sd="1" x="1"/>
+        <item t="data" sd="1" x="2"/>
+        <item t="data" sd="1" x="3"/>
+        <item t="data" sd="1" x="4"/>
+        <item t="default" sd="1"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1">
+      <items count="5">
+        <item t="data" sd="1" x="0"/>
+        <item t="data" sd="1" x="1"/>
+        <item t="data" sd="1" x="2"/>
+        <item t="data" sd="1" x="3"/>
+        <item t="default" sd="1"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1">
+      <items count="4">
+        <item t="data" sd="1" x="0"/>
+        <item t="data" sd="1" x="1"/>
+        <item t="data" sd="1" x="2"/>
+        <item t="default" sd="1"/>
+      </items>
+    </pivotField>
+    <pivotField showDropDowns="1" compact="1" outline="1" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="6">
+    <i t="data" r="0" i="0">
+      <x v="0"/>
+    </i>
+    <i t="data" r="0" i="0">
+      <x v="1"/>
+    </i>
+    <i t="data" r="0" i="0">
+      <x v="2"/>
+    </i>
+    <i t="data" r="0" i="0">
+      <x v="3"/>
+    </i>
+    <i t="data" r="0" i="0">
+      <x v="4"/>
+    </i>
+    <i t="grand" r="0" i="0">
+      <x v="0"/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="5"/>
+  </colFields>
+  <colItems count="4">
+    <i t="data" r="0" i="0">
+      <x v="0"/>
+    </i>
+    <i t="data" r="0" i="0">
+      <x v="1"/>
+    </i>
+    <i t="data" r="0" i="0">
+      <x v="2"/>
+    </i>
+    <i t="grand" r="0" i="0">
+      <x v="0"/>
+    </i>
+  </colItems>
+  <pageFields count="2">
+    <pageField fld="2" hier="-1"/>
+    <pageField fld="4" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Número de tareas" fld="0" subtotal="count" showDataAs="normal" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TablaTareas" displayName="TablaTareas" ref="A4:G44" headerRowCount="1">
+  <autoFilter ref="A4:G44"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="N.º"/>
+    <tableColumn id="2" name="Fecha de entrega"/>
+    <tableColumn id="3" name="Mes"/>
+    <tableColumn id="4" name="Asignatura"/>
+    <tableColumn id="5" name="Tipo de actividad"/>
+    <tableColumn id="6" name="Estado de entrega"/>
+    <tableColumn id="7" name="Calificación"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2351,6 +2891,228 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TABLA DINÁMICA: TAREAS POR ASIGNATURA Y ESTADO DE ENTREGA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Fuente: hoja REGISTRO DE TAREAS (tabla TablaTareas). Se actualiza al abrir el archivo; si cambias datos con el archivo abierto: clic derecho sobre la tabla dinámica &gt; Actualizar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>(Todas)</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Cómo usar los filtros</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tipo de actividad</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>(Todas)</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>1. Mes y Tipo de actividad (arriba de la tabla): elige uno o varios valores para filtrar todo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>2. Botones de Asignatura y Estado de entrega: muestran u ocultan asignaturas o estados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Número de tareas</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Estado de entrega</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>3. En la lista de campos puedes cambiar el cruce (por ejemplo, Promedio de Calificación por Mes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Asignatura</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Con retraso</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>No entregada</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Total general</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Comunicación oral y escrita</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologías de información</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Desarrollo humano</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Total general</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3182,11 +3944,11 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>4. Objetivo 2: entrega de tareas</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="30" customHeight="1">
+          <t>4. Objetivo 2: entrega de tareas (se calcula sola desde la hoja REGISTRO DE TAREAS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="40" customHeight="1">
       <c r="A45" s="7" t="inlineStr">
         <is>
           <t>Asignatura</t>
@@ -3194,17 +3956,17 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Tareas asignadas</t>
+          <t>Tareas asignadas (fórmula)</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Entregadas a tiempo</t>
+          <t>Entregadas a tiempo (fórmula)</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Entregadas con retraso</t>
+          <t>Entregadas con retraso (fórmula)</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -3228,13 +3990,16 @@
         <f>A37</f>
         <v>Matemáticas</v>
       </c>
-      <c r="B46" s="13" t="n">
+      <c r="B46" s="13">
+        <f>COUNTIF('REGISTRO DE TAREAS'!$D$5:$D$300,A46)</f>
         <v>10</v>
       </c>
-      <c r="C46" s="13" t="n">
+      <c r="C46" s="13">
+        <f>COUNTIFS('REGISTRO DE TAREAS'!$D$5:$D$300,A46,'REGISTRO DE TAREAS'!$F$5:$F$300,"A tiempo")</f>
         <v>7</v>
       </c>
-      <c r="D46" s="13" t="n">
+      <c r="D46" s="13">
+        <f>COUNTIFS('REGISTRO DE TAREAS'!$D$5:$D$300,A46,'REGISTRO DE TAREAS'!$F$5:$F$300,"Con retraso")</f>
         <v>2</v>
       </c>
       <c r="E46" s="13">
@@ -3255,13 +4020,16 @@
         <f>A38</f>
         <v>Comunicación oral y escrita</v>
       </c>
-      <c r="B47" s="13" t="n">
+      <c r="B47" s="13">
+        <f>COUNTIF('REGISTRO DE TAREAS'!$D$5:$D$300,A47)</f>
         <v>8</v>
       </c>
-      <c r="C47" s="13" t="n">
+      <c r="C47" s="13">
+        <f>COUNTIFS('REGISTRO DE TAREAS'!$D$5:$D$300,A47,'REGISTRO DE TAREAS'!$F$5:$F$300,"A tiempo")</f>
         <v>8</v>
       </c>
-      <c r="D47" s="13" t="n">
+      <c r="D47" s="13">
+        <f>COUNTIFS('REGISTRO DE TAREAS'!$D$5:$D$300,A47,'REGISTRO DE TAREAS'!$F$5:$F$300,"Con retraso")</f>
         <v>0</v>
       </c>
       <c r="E47" s="13">
@@ -3282,13 +4050,16 @@
         <f>A39</f>
         <v>Inglés</v>
       </c>
-      <c r="B48" s="13" t="n">
+      <c r="B48" s="13">
+        <f>COUNTIF('REGISTRO DE TAREAS'!$D$5:$D$300,A48)</f>
         <v>9</v>
       </c>
-      <c r="C48" s="13" t="n">
+      <c r="C48" s="13">
+        <f>COUNTIFS('REGISTRO DE TAREAS'!$D$5:$D$300,A48,'REGISTRO DE TAREAS'!$F$5:$F$300,"A tiempo")</f>
         <v>7</v>
       </c>
-      <c r="D48" s="13" t="n">
+      <c r="D48" s="13">
+        <f>COUNTIFS('REGISTRO DE TAREAS'!$D$5:$D$300,A48,'REGISTRO DE TAREAS'!$F$5:$F$300,"Con retraso")</f>
         <v>1</v>
       </c>
       <c r="E48" s="13">
@@ -3309,13 +4080,16 @@
         <f>A40</f>
         <v>Tecnologías de información</v>
       </c>
-      <c r="B49" s="13" t="n">
+      <c r="B49" s="13">
+        <f>COUNTIF('REGISTRO DE TAREAS'!$D$5:$D$300,A49)</f>
         <v>7</v>
       </c>
-      <c r="C49" s="13" t="n">
+      <c r="C49" s="13">
+        <f>COUNTIFS('REGISTRO DE TAREAS'!$D$5:$D$300,A49,'REGISTRO DE TAREAS'!$F$5:$F$300,"A tiempo")</f>
         <v>6</v>
       </c>
-      <c r="D49" s="13" t="n">
+      <c r="D49" s="13">
+        <f>COUNTIFS('REGISTRO DE TAREAS'!$D$5:$D$300,A49,'REGISTRO DE TAREAS'!$F$5:$F$300,"Con retraso")</f>
         <v>1</v>
       </c>
       <c r="E49" s="13">
@@ -3336,13 +4110,16 @@
         <f>A41</f>
         <v>Desarrollo humano</v>
       </c>
-      <c r="B50" s="13" t="n">
+      <c r="B50" s="13">
+        <f>COUNTIF('REGISTRO DE TAREAS'!$D$5:$D$300,A50)</f>
         <v>6</v>
       </c>
-      <c r="C50" s="13" t="n">
+      <c r="C50" s="13">
+        <f>COUNTIFS('REGISTRO DE TAREAS'!$D$5:$D$300,A50,'REGISTRO DE TAREAS'!$F$5:$F$300,"A tiempo")</f>
         <v>6</v>
       </c>
-      <c r="D50" s="13" t="n">
+      <c r="D50" s="13">
+        <f>COUNTIFS('REGISTRO DE TAREAS'!$D$5:$D$300,A50,'REGISTRO DE TAREAS'!$F$5:$F$300,"Con retraso")</f>
         <v>0</v>
       </c>
       <c r="E50" s="13">
@@ -4377,7 +5154,7 @@
       <formula>G46="Bajo rendimiento"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="9">
+  <dataValidations count="8">
     <dataValidation sqref="D21:D32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>60</formula2>
@@ -4397,10 +5174,6 @@
       <formula1>0</formula1>
       <formula2>10</formula2>
     </dataValidation>
-    <dataValidation sqref="B46:D50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
-      <formula1>0</formula1>
-      <formula2>200</formula2>
-    </dataValidation>
     <dataValidation sqref="B55:B60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Planeación,Curso,Currículum,Evento"</formula1>
     </dataValidation>
@@ -4418,7 +5191,1296 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>REGISTRO DE TAREAS (fuente de la tabla dinámica)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Una fila por tarea. Las tareas nuevas se escriben en la primera fila vacía debajo de la tabla (la tabla crece sola). La columna Mes se calcula sola. Los datos son de ejemplo: cámbialos por tus tareas reales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="37" t="inlineStr">
+        <is>
+          <t>N.º</t>
+        </is>
+      </c>
+      <c r="B4" s="37" t="inlineStr">
+        <is>
+          <t>Fecha de entrega</t>
+        </is>
+      </c>
+      <c r="C4" s="37" t="inlineStr">
+        <is>
+          <t>Mes</t>
+        </is>
+      </c>
+      <c r="D4" s="37" t="inlineStr">
+        <is>
+          <t>Asignatura</t>
+        </is>
+      </c>
+      <c r="E4" s="37" t="inlineStr">
+        <is>
+          <t>Tipo de actividad</t>
+        </is>
+      </c>
+      <c r="F4" s="37" t="inlineStr">
+        <is>
+          <t>Estado de entrega</t>
+        </is>
+      </c>
+      <c r="G4" s="37" t="inlineStr">
+        <is>
+          <t>Calificación</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="39" t="n">
+        <v>46267</v>
+      </c>
+      <c r="C5" s="38" t="str">
+        <f>IF(B5="","",CHOOSE(MONTH(B5),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F5" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G5" s="40" t="n">
+        <v>7.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="39" t="n">
+        <v>46268</v>
+      </c>
+      <c r="C6" s="38" t="str">
+        <f>IF(B6="","",CHOOSE(MONTH(B6),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Comunicación oral y escrita</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F6" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G6" s="40" t="n">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="39" t="n">
+        <v>46269</v>
+      </c>
+      <c r="C7" s="38" t="str">
+        <f>IF(B7="","",CHOOSE(MONTH(B7),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F7" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G7" s="40" t="n">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="39" t="n">
+        <v>46270</v>
+      </c>
+      <c r="C8" s="38" t="str">
+        <f>IF(B8="","",CHOOSE(MONTH(B8),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologías de información</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F8" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G8" s="40" t="n">
+        <v>8.699999999999999</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="39" t="n">
+        <v>46271</v>
+      </c>
+      <c r="C9" s="38" t="str">
+        <f>IF(B9="","",CHOOSE(MONTH(B9),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Desarrollo humano</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F9" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G9" s="40" t="n">
+        <v>9.300000000000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="39" t="n">
+        <v>46271</v>
+      </c>
+      <c r="C10" s="38" t="str">
+        <f>IF(B10="","",CHOOSE(MONTH(B10),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Ejercicios de repaso</t>
+        </is>
+      </c>
+      <c r="F10" s="38" t="inlineStr">
+        <is>
+          <t>Con retraso</t>
+        </is>
+      </c>
+      <c r="G10" s="40" t="n">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="38" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="39" t="n">
+        <v>46274</v>
+      </c>
+      <c r="C11" s="38" t="str">
+        <f>IF(B11="","",CHOOSE(MONTH(B11),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Comunicación oral y escrita</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Ejercicios de repaso</t>
+        </is>
+      </c>
+      <c r="F11" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G11" s="40" t="n">
+        <v>9.199999999999999</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="38" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="39" t="n">
+        <v>46274</v>
+      </c>
+      <c r="C12" s="38" t="str">
+        <f>IF(B12="","",CHOOSE(MONTH(B12),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>Ejercicios de repaso</t>
+        </is>
+      </c>
+      <c r="F12" s="38" t="inlineStr">
+        <is>
+          <t>Con retraso</t>
+        </is>
+      </c>
+      <c r="G12" s="40" t="n">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="38" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="39" t="n">
+        <v>46275</v>
+      </c>
+      <c r="C13" s="38" t="str">
+        <f>IF(B13="","",CHOOSE(MONTH(B13),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F13" s="38" t="inlineStr">
+        <is>
+          <t>No entregada</t>
+        </is>
+      </c>
+      <c r="G13" s="40" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="38" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="39" t="n">
+        <v>46276</v>
+      </c>
+      <c r="C14" s="38" t="str">
+        <f>IF(B14="","",CHOOSE(MONTH(B14),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologías de información</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Ejercicios de repaso</t>
+        </is>
+      </c>
+      <c r="F14" s="38" t="inlineStr">
+        <is>
+          <t>Con retraso</t>
+        </is>
+      </c>
+      <c r="G14" s="40" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="38" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="39" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C15" s="38" t="str">
+        <f>IF(B15="","",CHOOSE(MONTH(B15),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Desarrollo humano</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Ejercicios de repaso</t>
+        </is>
+      </c>
+      <c r="F15" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G15" s="40" t="n">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="38" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="39" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C16" s="38" t="str">
+        <f>IF(B16="","",CHOOSE(MONTH(B16),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F16" s="38" t="inlineStr">
+        <is>
+          <t>No entregada</t>
+        </is>
+      </c>
+      <c r="G16" s="40" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="38" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="39" t="n">
+        <v>46279</v>
+      </c>
+      <c r="C17" s="38" t="str">
+        <f>IF(B17="","",CHOOSE(MONTH(B17),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Reporte de lectura</t>
+        </is>
+      </c>
+      <c r="F17" s="38" t="inlineStr">
+        <is>
+          <t>Con retraso</t>
+        </is>
+      </c>
+      <c r="G17" s="40" t="n">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="38" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="39" t="n">
+        <v>46280</v>
+      </c>
+      <c r="C18" s="38" t="str">
+        <f>IF(B18="","",CHOOSE(MONTH(B18),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Comunicación oral y escrita</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F18" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G18" s="40" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="38" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="39" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C19" s="38" t="str">
+        <f>IF(B19="","",CHOOSE(MONTH(B19),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologías de información</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F19" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G19" s="40" t="n">
+        <v>9.300000000000001</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="38" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="39" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C20" s="38" t="str">
+        <f>IF(B20="","",CHOOSE(MONTH(B20),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="F20" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G20" s="40" t="n">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="38" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="39" t="n">
+        <v>46284</v>
+      </c>
+      <c r="C21" s="38" t="str">
+        <f>IF(B21="","",CHOOSE(MONTH(B21),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Reporte de lectura</t>
+        </is>
+      </c>
+      <c r="F21" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G21" s="40" t="n">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="38" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="39" t="n">
+        <v>46286</v>
+      </c>
+      <c r="C22" s="38" t="str">
+        <f>IF(B22="","",CHOOSE(MONTH(B22),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Comunicación oral y escrita</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Reporte de lectura</t>
+        </is>
+      </c>
+      <c r="F22" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G22" s="40" t="n">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="38" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="39" t="n">
+        <v>46287</v>
+      </c>
+      <c r="C23" s="38" t="str">
+        <f>IF(B23="","",CHOOSE(MONTH(B23),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Desarrollo humano</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F23" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G23" s="40" t="n">
+        <v>9.9</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="38" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="39" t="n">
+        <v>46287</v>
+      </c>
+      <c r="C24" s="38" t="str">
+        <f>IF(B24="","",CHOOSE(MONTH(B24),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F24" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G24" s="40" t="n">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="38" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="39" t="n">
+        <v>46288</v>
+      </c>
+      <c r="C25" s="38" t="str">
+        <f>IF(B25="","",CHOOSE(MONTH(B25),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologías de información</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>Reporte de lectura</t>
+        </is>
+      </c>
+      <c r="F25" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G25" s="40" t="n">
+        <v>8.699999999999999</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="38" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="39" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C26" s="38" t="str">
+        <f>IF(B26="","",CHOOSE(MONTH(B26),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="F26" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G26" s="40" t="n">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="38" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="39" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C27" s="38" t="str">
+        <f>IF(B27="","",CHOOSE(MONTH(B27),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>Ejercicios de repaso</t>
+        </is>
+      </c>
+      <c r="F27" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G27" s="40" t="n">
+        <v>7.3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="38" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="39" t="n">
+        <v>46292</v>
+      </c>
+      <c r="C28" s="38" t="str">
+        <f>IF(B28="","",CHOOSE(MONTH(B28),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Comunicación oral y escrita</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="F28" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G28" s="40" t="n">
+        <v>9.199999999999999</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="38" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="39" t="n">
+        <v>46294</v>
+      </c>
+      <c r="C29" s="38" t="str">
+        <f>IF(B29="","",CHOOSE(MONTH(B29),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F29" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G29" s="40" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="38" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="39" t="n">
+        <v>46294</v>
+      </c>
+      <c r="C30" s="38" t="str">
+        <f>IF(B30="","",CHOOSE(MONTH(B30),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologías de información</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="F30" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G30" s="40" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="38" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="39" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C31" s="38" t="str">
+        <f>IF(B31="","",CHOOSE(MONTH(B31),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Desarrollo humano</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Reporte de lectura</t>
+        </is>
+      </c>
+      <c r="F31" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G31" s="40" t="n">
+        <v>9.300000000000001</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="38" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="39" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C32" s="38" t="str">
+        <f>IF(B32="","",CHOOSE(MONTH(B32),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Septiembre</v>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F32" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G32" s="40" t="n">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="38" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="39" t="n">
+        <v>46298</v>
+      </c>
+      <c r="C33" s="38" t="str">
+        <f>IF(B33="","",CHOOSE(MONTH(B33),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Octubre</v>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>Comunicación oral y escrita</t>
+        </is>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F33" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G33" s="40" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="38" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="39" t="n">
+        <v>46299</v>
+      </c>
+      <c r="C34" s="38" t="str">
+        <f>IF(B34="","",CHOOSE(MONTH(B34),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Octubre</v>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>Ejercicios de repaso</t>
+        </is>
+      </c>
+      <c r="F34" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G34" s="40" t="n">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="38" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="39" t="n">
+        <v>46299</v>
+      </c>
+      <c r="C35" s="38" t="str">
+        <f>IF(B35="","",CHOOSE(MONTH(B35),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Octubre</v>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>Reporte de lectura</t>
+        </is>
+      </c>
+      <c r="F35" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G35" s="40" t="n">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="38" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="39" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C36" s="38" t="str">
+        <f>IF(B36="","",CHOOSE(MONTH(B36),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Octubre</v>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologías de información</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F36" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G36" s="40" t="n">
+        <v>9.300000000000001</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="38" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="39" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C37" s="38" t="str">
+        <f>IF(B37="","",CHOOSE(MONTH(B37),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Octubre</v>
+      </c>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t>Desarrollo humano</t>
+        </is>
+      </c>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="F37" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G37" s="40" t="n">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="38" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="39" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C38" s="38" t="str">
+        <f>IF(B38="","",CHOOSE(MONTH(B38),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Octubre</v>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="F38" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G38" s="40" t="n">
+        <v>7.3</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="38" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="39" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C39" s="38" t="str">
+        <f>IF(B39="","",CHOOSE(MONTH(B39),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Octubre</v>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>Comunicación oral y escrita</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>Ejercicios de repaso</t>
+        </is>
+      </c>
+      <c r="F39" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G39" s="40" t="n">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="38" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="39" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C40" s="38" t="str">
+        <f>IF(B40="","",CHOOSE(MONTH(B40),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Octubre</v>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F40" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G40" s="40" t="n">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="39" t="n">
+        <v>46306</v>
+      </c>
+      <c r="C41" s="38" t="str">
+        <f>IF(B41="","",CHOOSE(MONTH(B41),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Octubre</v>
+      </c>
+      <c r="D41" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologías de información</t>
+        </is>
+      </c>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>Ejercicios de repaso</t>
+        </is>
+      </c>
+      <c r="F41" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G41" s="40" t="n">
+        <v>8.699999999999999</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="38" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="39" t="n">
+        <v>46309</v>
+      </c>
+      <c r="C42" s="38" t="str">
+        <f>IF(B42="","",CHOOSE(MONTH(B42),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Octubre</v>
+      </c>
+      <c r="D42" s="11" t="inlineStr">
+        <is>
+          <t>Inglés</t>
+        </is>
+      </c>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>Reporte de lectura</t>
+        </is>
+      </c>
+      <c r="F42" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G42" s="40" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="38" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="39" t="n">
+        <v>46310</v>
+      </c>
+      <c r="C43" s="38" t="str">
+        <f>IF(B43="","",CHOOSE(MONTH(B43),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Octubre</v>
+      </c>
+      <c r="D43" s="11" t="inlineStr">
+        <is>
+          <t>Comunicación oral y escrita</t>
+        </is>
+      </c>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F43" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G43" s="40" t="n">
+        <v>9.199999999999999</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="38" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="39" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C44" s="38" t="str">
+        <f>IF(B44="","",CHOOSE(MONTH(B44),"Enero","Febrero","Marzo","Abril","Mayo","Junio","Julio","Agosto","Septiembre","Octubre","Noviembre","Diciembre"))</f>
+        <v>Octubre</v>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>Desarrollo humano</t>
+        </is>
+      </c>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="F44" s="38" t="inlineStr">
+        <is>
+          <t>A tiempo</t>
+        </is>
+      </c>
+      <c r="G44" s="40" t="n">
+        <v>9.9</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation sqref="D5:D300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>DATOS!$A$37:$A$41</formula1>
+    </dataValidation>
+    <dataValidation sqref="E5:E300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Tarea,Ejercicios de repaso,Reporte de lectura,Proyecto"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F5:F300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"A tiempo,Con retraso,No entregada"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G5:G300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>10</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>